<commit_message>
Clarified instructions and explanation of regex
</commit_message>
<xml_diff>
--- a/solution_conference_talks_data.xlsx
+++ b/solution_conference_talks_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,452 +417,452 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Speaker_Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Talk_Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Kicker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Matthew</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Mark</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Luke</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>John</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Acts</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Romans</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>1 Corinthians</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>2 Corinthians</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Galatians</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Ephesians</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Philippians</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Colossians</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>1 Thessalonians</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>2 Thessalonians</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>1 Timothy</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>2 Timothy</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Titus</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Philemon</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Hebrews</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>James</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>1 Peter</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>2 Peter</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>1 John</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>2 John</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>3 John</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Jude</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Revelation</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Genesis</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Exodus</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Leviticus</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Numbers</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Deuteronomy</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Joshua</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Judges</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Ruth</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>1 Samuel</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>2 Samuel</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>1 Kings</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>2 Kings</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>1 Chronicles</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>2 Chronicles</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Ezra</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Nehemiah</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>Esther</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>Job</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>Psalm</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>Proverbs</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>Ecclesiastes</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>Song of Solomon</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>Isaiah</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>Jeremiah</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>Lamentations</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>Ezekiel</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>Daniel</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>Hosea</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>Joel</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>Amos</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>Obadiah</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>Jonah</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>Micah</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>Nahum</t>
         </is>
       </c>
-      <c r="BM1" s="1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>Habakkuk</t>
         </is>
       </c>
-      <c r="BN1" s="1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>Zephaniah</t>
         </is>
       </c>
-      <c r="BO1" s="1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>Haggai</t>
         </is>
       </c>
-      <c r="BP1" s="1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>Zechariah</t>
         </is>
       </c>
-      <c r="BQ1" s="1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>Malachi</t>
         </is>
       </c>
-      <c r="BR1" s="1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>1 Nephi</t>
         </is>
       </c>
-      <c r="BS1" s="1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>2 Nephi</t>
         </is>
       </c>
-      <c r="BT1" s="1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>Jacob</t>
         </is>
       </c>
-      <c r="BU1" s="1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>Enos</t>
         </is>
       </c>
-      <c r="BV1" s="1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>Jarom</t>
         </is>
       </c>
-      <c r="BW1" s="1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>Omni</t>
         </is>
       </c>
-      <c r="BX1" s="1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>Words of Mormon</t>
         </is>
       </c>
-      <c r="BY1" s="1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>Mosiah</t>
         </is>
       </c>
-      <c r="BZ1" s="1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>Alma</t>
         </is>
       </c>
-      <c r="CA1" s="1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>Helaman</t>
         </is>
       </c>
-      <c r="CB1" s="1" t="inlineStr">
+      <c r="CB1" t="inlineStr">
         <is>
           <t>3 Nephi</t>
         </is>
       </c>
-      <c r="CC1" s="1" t="inlineStr">
+      <c r="CC1" t="inlineStr">
         <is>
           <t>4 Nephi</t>
         </is>
       </c>
-      <c r="CD1" s="1" t="inlineStr">
+      <c r="CD1" t="inlineStr">
         <is>
           <t>Mormon</t>
         </is>
       </c>
-      <c r="CE1" s="1" t="inlineStr">
+      <c r="CE1" t="inlineStr">
         <is>
           <t>Ether</t>
         </is>
       </c>
-      <c r="CF1" s="1" t="inlineStr">
+      <c r="CF1" t="inlineStr">
         <is>
           <t>Moroni</t>
         </is>
       </c>
-      <c r="CG1" s="1" t="inlineStr">
+      <c r="CG1" t="inlineStr">
         <is>
           <t>Doctrine and Covenants</t>
         </is>
       </c>
-      <c r="CH1" s="1" t="inlineStr">
+      <c r="CH1" t="inlineStr">
         <is>
           <t>Moses</t>
         </is>
       </c>
-      <c r="CI1" s="1" t="inlineStr">
+      <c r="CI1" t="inlineStr">
         <is>
           <t>Abraham</t>
         </is>
       </c>
-      <c r="CJ1" s="1" t="inlineStr">
+      <c r="CJ1" t="inlineStr">
         <is>
           <t>Joseph Smith—Matthew</t>
         </is>
       </c>
-      <c r="CK1" s="1" t="inlineStr">
+      <c r="CK1" t="inlineStr">
         <is>
           <t>Joseph Smith—History</t>
         </is>
       </c>
-      <c r="CL1" s="1" t="inlineStr">
+      <c r="CL1" t="inlineStr">
         <is>
           <t>Articles of Faith</t>
         </is>
@@ -1184,7 +1172,7 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -3077,7 +3065,7 @@
         <v>0</v>
       </c>
       <c r="CD9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CE9" t="n">
         <v>0</v>
@@ -3199,7 +3187,7 @@
         <v>0</v>
       </c>
       <c r="AD10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
@@ -3755,7 +3743,7 @@
         <v>0</v>
       </c>
       <c r="AD12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AE12" t="n">
         <v>0</v>
@@ -3881,7 +3869,7 @@
         <v>2</v>
       </c>
       <c r="BT12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BU12" t="n">
         <v>0</v>
@@ -3911,7 +3899,7 @@
         <v>0</v>
       </c>
       <c r="CD12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CE12" t="n">
         <v>0</v>
@@ -4189,7 +4177,7 @@
         <v>0</v>
       </c>
       <c r="CD13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CE13" t="n">
         <v>0</v>
@@ -4311,7 +4299,7 @@
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE14" t="n">
         <v>0</v>
@@ -4568,7 +4556,7 @@
         <v>0</v>
       </c>
       <c r="W15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X15" t="n">
         <v>0</v>
@@ -4745,7 +4733,7 @@
         <v>0</v>
       </c>
       <c r="CD15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="CE15" t="n">
         <v>0</v>
@@ -5011,7 +4999,7 @@
         <v>2</v>
       </c>
       <c r="BZ16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CA16" t="n">
         <v>0</v>
@@ -5232,7 +5220,7 @@
         <v>0</v>
       </c>
       <c r="BG17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BH17" t="n">
         <v>0</v>
@@ -5468,7 +5456,7 @@
         <v>0</v>
       </c>
       <c r="AS18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT18" t="n">
         <v>0</v>
@@ -7022,7 +7010,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H24" t="n">
         <v>4</v>
@@ -7217,7 +7205,7 @@
         <v>0</v>
       </c>
       <c r="BT24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BU24" t="n">
         <v>0</v>
@@ -7247,7 +7235,7 @@
         <v>0</v>
       </c>
       <c r="CD24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CE24" t="n">
         <v>0</v>
@@ -7513,7 +7501,7 @@
         <v>0</v>
       </c>
       <c r="BZ25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="CA25" t="n">
         <v>1</v>
@@ -7776,7 +7764,7 @@
         <v>0</v>
       </c>
       <c r="BU26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BV26" t="n">
         <v>0</v>
@@ -7803,7 +7791,7 @@
         <v>0</v>
       </c>
       <c r="CD26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CE26" t="n">
         <v>2</v>
@@ -8792,7 +8780,7 @@
         <v>0</v>
       </c>
       <c r="AO30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP30" t="n">
         <v>0</v>
@@ -8813,7 +8801,7 @@
         <v>0</v>
       </c>
       <c r="AV30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW30" t="n">
         <v>0</v>
@@ -8855,7 +8843,7 @@
         <v>0</v>
       </c>
       <c r="BJ30" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="BK30" t="n">
         <v>0</v>
@@ -8876,7 +8864,7 @@
         <v>0</v>
       </c>
       <c r="BQ30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BR30" t="n">
         <v>1</v>
@@ -8915,7 +8903,7 @@
         <v>0</v>
       </c>
       <c r="CD30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CE30" t="n">
         <v>0</v>
@@ -9016,7 +9004,7 @@
         <v>0</v>
       </c>
       <c r="W31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X31" t="n">
         <v>0</v>
@@ -9294,7 +9282,7 @@
         <v>0</v>
       </c>
       <c r="W32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X32" t="n">
         <v>0</v>
@@ -9339,7 +9327,7 @@
         <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -9384,7 +9372,7 @@
         <v>0</v>
       </c>
       <c r="BA32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB32" t="n">
         <v>0</v>
@@ -9471,7 +9459,7 @@
         <v>0</v>
       </c>
       <c r="CD32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CE32" t="n">
         <v>1</v>
@@ -9593,7 +9581,7 @@
         <v>0</v>
       </c>
       <c r="AD33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE33" t="n">
         <v>0</v>

</xml_diff>